<commit_message>
Add spelling changes to TCs
</commit_message>
<xml_diff>
--- a/Test-Cases/Swag Labs test suit.xlsx
+++ b/Test-Cases/Swag Labs test suit.xlsx
@@ -9,13 +9,15 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="75" windowWidth="18195" windowHeight="11820" activeTab="4"/>
+    <workbookView xWindow="480" yWindow="75" windowWidth="18195" windowHeight="11820" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenarious" sheetId="1" r:id="rId1"/>
     <sheet name="Login" sheetId="2" r:id="rId2"/>
     <sheet name="Logout" sheetId="3" r:id="rId7"/>
     <sheet name="Add to cart" sheetId="4" r:id="rId8"/>
+    <sheet name="Remove Product" sheetId="7" r:id="rId3"/>
+    <sheet name="Your Cart" sheetId="6" r:id="rId10"/>
     <sheet name="Checkout" sheetId="5" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
@@ -541,12 +543,208 @@
     <t>The user cannot complete the checkout process with an empty cart.
 The application keeps the user on the Cart page or prevents further checkout steps.</t>
   </si>
+  <si>
+    <t>Validate successful getting back to Products page from the cart</t>
+  </si>
+  <si>
+    <t>1. Go to the Shopping Cart by clicking the cart icon (top right corner)</t>
+  </si>
+  <si>
+    <t>1. Go to the Shopping Cart by clicking the cart icon (top right corner)
+2. Click 'Continue Shopping' button</t>
+  </si>
+  <si>
+    <t>1. The user is returned to the Products page</t>
+  </si>
+  <si>
+    <t>TC2</t>
+  </si>
+  <si>
+    <t>TS8</t>
+  </si>
+  <si>
+    <t>Validate successful navigation back to Products page from the cart</t>
+  </si>
+  <si>
+    <t>Validate successful navigation to the specific Products from the cart</t>
+  </si>
+  <si>
+    <t>Validate successful navigation to the specific Product's details page from the cart</t>
+  </si>
+  <si>
+    <t>1. Go to the Shopping Cart by clicking the cart icon (top right corner)
+2. Click on the title of the added product</t>
+  </si>
+  <si>
+    <t>The user is returned to the Products page</t>
+  </si>
+  <si>
+    <t>The user is navigated successfully to the Product's details page</t>
+  </si>
+  <si>
+    <t>Validate successful removal of a specific Product from the cart</t>
+  </si>
+  <si>
+    <t>1. Go to the Shopping Cart by clicking the cart icon (top right corner)
+2. Click the 'Remove' button of the added product</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>z</t>
+  </si>
+  <si>
+    <t>TC0033</t>
+  </si>
+  <si>
+    <t>Validate successful removal of all Products from the cart</t>
+  </si>
+  <si>
+    <t>1. The user is logged in and on the Products page (https://www.saucedemo.com/inventory.html)
+2. At least two products has been added to the shopping cart</t>
+  </si>
+  <si>
+    <t>1. Go to the Shopping Cart by clicking the cart icon (top right corner)
+2. Click the 'Remove' button for all added product</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. The selected products are removed from the shopping cart
+2. The number displayed on the shopping cart icon decreases accordingly
+3. The cart is empty </t>
+  </si>
+  <si>
+    <t>1. Go to the Shopping Cart by clicking the cart icon (top right corner)
+2. Click the 'Remove' button for the added product</t>
+  </si>
+  <si>
+    <t>Verify that a specific product can be removed from the shopping cart</t>
+  </si>
+  <si>
+    <t>1. User is logged in and on the Products page (https://www.saucedemo.com/inventory.html)
+2. At least one product is added to the shopping cart</t>
+  </si>
+  <si>
+    <t>1. Click on the Shopping Cart icon (top-right corner)
+2. Click the 'Remove' button for the added product</t>
+  </si>
+  <si>
+    <t>1. The selected product is removed from the cart
+2. The cart badge counter decreases by 1 accordingly</t>
+  </si>
+  <si>
+    <t>Verify that all products can be removed from the shopping cart</t>
+  </si>
+  <si>
+    <t>1. The user is logged in and on the Products page (https://www.saucedemo.com/inventory.html)
+2. At least two products are added to the shopping cart</t>
+  </si>
+  <si>
+    <t>1. Click on the Shopping Cart icon (top-right corner)
+2. For each product in the cart, click the 'Remove' button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. All products are removed from the shopping cart
+2. The number displayed on the shopping cart icon decreases accordingly
+3. The cart is empty </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. All products are removed from the shopping cart
+2. The cart badge counter is cleared (disappears)
+3. The cart is empty </t>
+  </si>
+  <si>
+    <t>Verify navigation back to Products page from the shopping cart</t>
+  </si>
+  <si>
+    <t>1. Click on the Shopping Cart icon (top-right corner)
+2. Click 'Continue Shopping' button</t>
+  </si>
+  <si>
+    <t>User is redirected back to the Products page
+Products listing page is displayed correctly</t>
+  </si>
+  <si>
+    <t>Verify navigation to Products deatils page from the shopping cart</t>
+  </si>
+  <si>
+    <t>1. The user is logged in and on the Products page (https://www.saucedemo.com/inventory.html)
+2. At least one product is added to the shopping cart</t>
+  </si>
+  <si>
+    <t>1. Click on the Shopping Cart icon (top-right corner)
+2. Click on the product name(title) button in the cart</t>
+  </si>
+  <si>
+    <t>User is redirected to the correct Product Details page
+Products details match the selected item</t>
+  </si>
+  <si>
+    <t>1. Click the 'Remove' button for a product on the Products page
+2. Go to the Shopping Cart by clicking the cart icon (top right corner)</t>
+  </si>
+  <si>
+    <t>1. The selected product is removed from the cart
+2. The shopping cart badge counter decreases accordingly</t>
+  </si>
+  <si>
+    <t>Verify that a Product can be successfully added to the cart by a Logged-in User</t>
+  </si>
+  <si>
+    <t>1. Click 'Add to cart' button for any product
+2. Go to the Shopping Cart by clicking the cart icon (top right corner)</t>
+  </si>
+  <si>
+    <t>1. Click 'Add to cart' button for any product
+2. Click on the Shopping Cart icon (top-right corner)</t>
+  </si>
+  <si>
+    <t>Verify Error Message when accessing the Product page without login</t>
+  </si>
+  <si>
+    <t>User is not logged in</t>
+  </si>
+  <si>
+    <t>1. Error message is displayed: "Epic sadface: You can only access '/inventory.html' when you are logged in." 
+2. User remains on the Login page</t>
+  </si>
+  <si>
+    <t>Verify successful Logout for standard user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click on the hamburger menu (top-left corner)
+2. Click 'Logout' </t>
+  </si>
+  <si>
+    <t>Verify successful login with valid credentials</t>
+  </si>
+  <si>
+    <t>1. Enter standart_user in the Username field
+2. Enter secret_sauce in the Password field
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>1. The user is logged in successfully
+2. Products page is displayed</t>
+  </si>
+  <si>
+    <t>Verify unsuccessful login for a locked-out user</t>
+  </si>
+  <si>
+    <t>1. Enter locked_out_user in the Username field
+2. Enter secret_sauce in the Password field
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>1. The user is not logged
+2. Error message is displayed: 'Epic sadface: Sorry, this user has been locked out.'</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -562,8 +760,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FFFFFFFF"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FFF2F2F2"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -620,6 +832,11 @@
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -633,7 +850,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" xfId="0"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="2" applyFill="1" xfId="0"/>
@@ -658,6 +875,10 @@
     </xf>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="10" applyFill="1" xfId="0"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="11" applyFill="1" xfId="0"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="2" applyFont="1" fillId="10" applyFill="1" xfId="0"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="3" applyFont="1" fillId="10" applyFill="1" xfId="0"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="2" applyFont="1" fillId="12" applyFill="1" xfId="0"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="2" applyFont="1" fillId="11" applyFill="1" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1125,19 +1346,19 @@
         <v>16</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>86</v>
+        <v>197</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>70</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>71</v>
+        <v>198</v>
       </c>
       <c r="F2" s="11" t="s">
         <v>45</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>73</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" ht="69">
@@ -1148,22 +1369,139 @@
         <v>16</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>70</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>77</v>
+        <v>201</v>
       </c>
       <c r="F3" s="11" t="s">
         <v>57</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>64</v>
+        <v>202</v>
+      </c>
+      <c r="I3" s="19"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25" outlineLevelRow="0" outlineLevelCol="0" defaultColWidth="8.609375"/>
+  <cols>
+    <col min="1" max="1" width="12.5078125" customWidth="1"/>
+    <col min="2" max="2" width="11.02734375" customWidth="1"/>
+    <col min="3" max="3" width="38.47265625" customWidth="1"/>
+    <col min="4" max="4" width="29.86328125" customWidth="1"/>
+    <col min="5" max="5" width="16.41015625" customWidth="1"/>
+    <col min="6" max="6" width="16.27734375" customWidth="1"/>
+    <col min="7" max="7" width="26.90234375" customWidth="1"/>
+    <col min="8" max="8" width="12.10546875" customWidth="1"/>
+    <col min="9" max="9" width="18.5625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" ht="123">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="3" ht="96">
+      <c r="A3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4" ht="96">
+      <c r="A4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -1216,7 +1554,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" ht="109.5">
+    <row r="2" ht="69">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -1224,13 +1562,13 @@
         <v>18</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>90</v>
+        <v>195</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>91</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>92</v>
+        <v>196</v>
       </c>
       <c r="F2" s="11" t="s">
         <v>67</v>
@@ -1296,7 +1634,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" ht="123">
+    <row r="2" ht="96">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -1304,13 +1642,13 @@
         <v>20</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>117</v>
+        <v>189</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>118</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>119</v>
+        <v>191</v>
       </c>
       <c r="F2" s="11" t="s">
         <v>45</v>
@@ -1327,9 +1665,11 @@
         <v>20</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="D3" s="11"/>
+        <v>192</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>193</v>
+      </c>
       <c r="E3" s="11" t="s">
         <v>122</v>
       </c>
@@ -1337,31 +1677,15 @@
         <v>67</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="4" ht="123">
-      <c r="A4" t="s">
-        <v>108</v>
-      </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>132</v>
-      </c>
+        <v>194</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1467,4 +1791,100 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25" outlineLevelRow="0" outlineLevelCol="0" defaultColWidth="8.609375"/>
+  <cols>
+    <col min="1" max="1" width="12.5078125" customWidth="1"/>
+    <col min="2" max="2" width="11.02734375" customWidth="1"/>
+    <col min="3" max="3" width="38.47265625" customWidth="1"/>
+    <col min="4" max="4" width="29.86328125" customWidth="1"/>
+    <col min="5" max="5" width="13.44921875" customWidth="1"/>
+    <col min="6" max="6" width="16.27734375" customWidth="1"/>
+    <col min="7" max="7" width="26.90234375" customWidth="1"/>
+    <col min="8" max="8" width="12.10546875" customWidth="1"/>
+    <col min="9" max="9" width="18.5625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" ht="109.5">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="3" ht="123">
+      <c r="A3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>186</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add spelling changes to TCs and added new TCs
</commit_message>
<xml_diff>
--- a/Test-Cases/Swag Labs test suit.xlsx
+++ b/Test-Cases/Swag Labs test suit.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="75" windowWidth="18195" windowHeight="11820" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="75" windowWidth="18195" windowHeight="11820" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenarious" sheetId="1" r:id="rId1"/>
@@ -738,6 +738,12 @@
   <si>
     <t>1. The user is not logged
 2. Error message is displayed: 'Epic sadface: Sorry, this user has been locked out.'</t>
+  </si>
+  <si>
+    <t>1. The user is on the login page of Sauce Demo (https://www.saucedemo.com)</t>
+  </si>
+  <si>
+    <t>Verify navigation to Products details page from the shopping cart</t>
   </si>
 </sst>
 </file>
@@ -1349,7 +1355,7 @@
         <v>197</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>70</v>
+        <v>203</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>198</v>
@@ -1372,7 +1378,7 @@
         <v>200</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>70</v>
+        <v>203</v>
       </c>
       <c r="E3" s="11" t="s">
         <v>201</v>
@@ -1869,7 +1875,7 @@
         <v>31</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>183</v>
+        <v>204</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>184</v>

</xml_diff>